<commit_message>
Update GhostIQ MLB live data
</commit_message>
<xml_diff>
--- a/outputs/daily/hr_rankings_2026-10-01.xlsx
+++ b/outputs/daily/hr_rankings_2026-10-01.xlsx
@@ -840,7 +840,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -1196,7 +1196,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -1552,7 +1552,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -1866,7 +1866,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -2222,7 +2222,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -2578,7 +2578,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -2934,7 +2934,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -3248,7 +3248,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -3604,7 +3604,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -3918,7 +3918,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -4232,7 +4232,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -4546,7 +4546,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -4860,7 +4860,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -5174,7 +5174,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -5488,7 +5488,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -5802,7 +5802,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -6116,7 +6116,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -6430,7 +6430,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -7150,7 +7150,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -7506,7 +7506,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -7862,7 +7862,7 @@
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -8176,7 +8176,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -8532,7 +8532,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -8888,7 +8888,7 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -9244,7 +9244,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -9558,7 +9558,7 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -9914,7 +9914,7 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -10228,7 +10228,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -10542,7 +10542,7 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -10856,7 +10856,7 @@
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -11170,7 +11170,7 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -11484,7 +11484,7 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -11798,7 +11798,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -12112,7 +12112,7 @@
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -12426,7 +12426,7 @@
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -12740,7 +12740,7 @@
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Pre-Game</t>
+          <t>Warmup</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">

</xml_diff>